<commit_message>
feat(coverage): CIGA dual evidence unlocks open_tenders 100% coverage
- project_ciga_dual_evidence writes coverage_evidence for municipal entities
- VPS dual gate PASS: 1093/1093, 0 unknown, freshness 1093
- verify-production 8/9; only soak_7d remains (calendar)
- fix DOM-SC month sort for recent packages
</commit_message>
<xml_diff>
--- a/artifacts/campaigns/OPEN-TENDERS-OPERATIONAL-DECISION-CYCLE-01/weekly-offline-rc/extra_weekly_pack.xlsx
+++ b/artifacts/campaigns/OPEN-TENDERS-OPERATIONAL-DECISION-CYCLE-01/weekly-offline-rc/extra_weekly_pack.xlsx
@@ -443,7 +443,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>weekly-20260723T231127Z-ab75580fcc</t>
+          <t>weekly-20260723T234219Z-b1c82d43ce</t>
         </is>
       </c>
     </row>
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260723T231127Z-3b479073</t>
+          <t>col-extra-weekly-20260723T234219Z-d1868440</t>
         </is>
       </c>
     </row>
@@ -467,7 +467,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-23T23:11:27Z</t>
+          <t>2026-07-23T23:42:19Z</t>
         </is>
       </c>
     </row>
@@ -479,7 +479,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ee4bb12b49281622cbf15ddc24f7741c00060e9e</t>
+          <t>6db0a6987c425bcd3bdcdeb97bc0230ddfb3c41b</t>
         </is>
       </c>
     </row>
@@ -844,12 +844,12 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260723T231127Z-3b479073</t>
+          <t>col-extra-weekly-20260723T234219Z-d1868440</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260723T231128Z-a68b48c8d2</t>
+          <t>collect-pncp_opportunities-20260723T234221Z-10d16aeb86</t>
         </is>
       </c>
       <c r="AH2" t="inlineStr">
@@ -1009,12 +1009,12 @@
       </c>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260723T231127Z-3b479073</t>
+          <t>col-extra-weekly-20260723T234219Z-d1868440</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260723T231128Z-a68b48c8d2</t>
+          <t>collect-pncp_opportunities-20260723T234221Z-10d16aeb86</t>
         </is>
       </c>
       <c r="AH3" t="inlineStr">
@@ -1174,12 +1174,12 @@
       </c>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260723T231127Z-3b479073</t>
+          <t>col-extra-weekly-20260723T234219Z-d1868440</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260723T231128Z-a68b48c8d2</t>
+          <t>collect-pncp_opportunities-20260723T234221Z-10d16aeb86</t>
         </is>
       </c>
       <c r="AH4" t="inlineStr">
@@ -1339,12 +1339,12 @@
       </c>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260723T231127Z-3b479073</t>
+          <t>col-extra-weekly-20260723T234219Z-d1868440</t>
         </is>
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260723T231128Z-a68b48c8d2</t>
+          <t>collect-pncp_opportunities-20260723T234221Z-10d16aeb86</t>
         </is>
       </c>
       <c r="AH5" t="inlineStr">
@@ -1479,7 +1479,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260723T231127Z-3b479073</t>
+          <t>col-extra-weekly-20260723T234219Z-d1868440</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260723T231127Z-3b479073</t>
+          <t>col-extra-weekly-20260723T234219Z-d1868440</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260723T231127Z-3b479073</t>
+          <t>col-extra-weekly-20260723T234219Z-d1868440</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1590,7 +1590,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260723T231127Z-3b479073</t>
+          <t>col-extra-weekly-20260723T234219Z-d1868440</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0.11</t>
+          <t>0.62</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>3.02</t>
+          <t>3.53</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>

</xml_diff>

<commit_message>
docs(ops): re-verify 8/9 PASS after VPS snapshot integrity refresh (BLOCKED soak only)
</commit_message>
<xml_diff>
--- a/artifacts/campaigns/OPEN-TENDERS-OPERATIONAL-DECISION-CYCLE-01/weekly-offline-rc/extra_weekly_pack.xlsx
+++ b/artifacts/campaigns/OPEN-TENDERS-OPERATIONAL-DECISION-CYCLE-01/weekly-offline-rc/extra_weekly_pack.xlsx
@@ -443,7 +443,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>weekly-20260723T234219Z-b1c82d43ce</t>
+          <t>weekly-20260724T001238Z-cd7bad9648</t>
         </is>
       </c>
     </row>
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260723T234219Z-d1868440</t>
+          <t>col-extra-weekly-20260724T001238Z-ee77044c</t>
         </is>
       </c>
     </row>
@@ -467,7 +467,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-23T23:42:19Z</t>
+          <t>2026-07-24T00:12:38Z</t>
         </is>
       </c>
     </row>
@@ -479,7 +479,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>6db0a6987c425bcd3bdcdeb97bc0230ddfb3c41b</t>
+          <t>68752046e9d93ecb8e37a8111ed709261f3da595</t>
         </is>
       </c>
     </row>
@@ -844,12 +844,12 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260723T234219Z-d1868440</t>
+          <t>col-extra-weekly-20260724T001238Z-ee77044c</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260723T234221Z-10d16aeb86</t>
+          <t>collect-pncp_opportunities-20260724T001240Z-1060734f2b</t>
         </is>
       </c>
       <c r="AH2" t="inlineStr">
@@ -1009,12 +1009,12 @@
       </c>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260723T234219Z-d1868440</t>
+          <t>col-extra-weekly-20260724T001238Z-ee77044c</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260723T234221Z-10d16aeb86</t>
+          <t>collect-pncp_opportunities-20260724T001240Z-1060734f2b</t>
         </is>
       </c>
       <c r="AH3" t="inlineStr">
@@ -1174,12 +1174,12 @@
       </c>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260723T234219Z-d1868440</t>
+          <t>col-extra-weekly-20260724T001238Z-ee77044c</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260723T234221Z-10d16aeb86</t>
+          <t>collect-pncp_opportunities-20260724T001240Z-1060734f2b</t>
         </is>
       </c>
       <c r="AH4" t="inlineStr">
@@ -1339,12 +1339,12 @@
       </c>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260723T234219Z-d1868440</t>
+          <t>col-extra-weekly-20260724T001238Z-ee77044c</t>
         </is>
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260723T234221Z-10d16aeb86</t>
+          <t>collect-pncp_opportunities-20260724T001240Z-1060734f2b</t>
         </is>
       </c>
       <c r="AH5" t="inlineStr">
@@ -1479,7 +1479,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260723T234219Z-d1868440</t>
+          <t>col-extra-weekly-20260724T001238Z-ee77044c</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260723T234219Z-d1868440</t>
+          <t>col-extra-weekly-20260724T001238Z-ee77044c</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260723T234219Z-d1868440</t>
+          <t>col-extra-weekly-20260724T001238Z-ee77044c</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1590,7 +1590,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260723T234219Z-d1868440</t>
+          <t>col-extra-weekly-20260724T001238Z-ee77044c</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0.62</t>
+          <t>1.13</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>3.53</t>
+          <t>4.04</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>

</xml_diff>